<commit_message>
update test to support approval flow
</commit_message>
<xml_diff>
--- a/api/fixtures/digital-consent-employee-id-import-approval.xlsx
+++ b/api/fixtures/digital-consent-employee-id-import-approval.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Documents/SH Test Data/Digital Consent/QA - Digital Consent Employee ID/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Workspace/qa-tests/api/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{816F40E6-7D88-DC42-9B28-D2D87B2804B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E852A9-283C-694C-9943-90919E5528C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24000" yWindow="500" windowWidth="14400" windowHeight="16360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="500" windowWidth="14400" windowHeight="16380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -243,7 +243,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -277,12 +277,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -296,6 +305,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -663,6 +673,7 @@
     <col min="27" max="27" width="11.5" customWidth="1"/>
     <col min="28" max="28" width="15.1640625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="0" hidden="1" customWidth="1"/>
     <col min="31" max="16384" width="8.83203125" hidden="1"/>
   </cols>
   <sheetData>
@@ -885,17 +896,23 @@
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:29" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="H6" s="7"/>
+    </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="Z7" s="4"/>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="F8" s="7"/>
+    </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.2"/>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2"/>
     <row r="11" spans="1:29" x14ac:dyDescent="0.2"/>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2"/>
     <row r="13" spans="1:29" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="G14" s="7"/>
+    </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -909,6 +926,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="e72a1ac6-4952-47dd-a4df-3296734776f1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f34ab2e2-b096-4083-affb-0a831dd0603a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A840765D86F0EA419C465DF1840FAAF8" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7889e1239fba0097d9d590902a836c0f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f34ab2e2-b096-4083-affb-0a831dd0603a" xmlns:ns3="e72a1ac6-4952-47dd-a4df-3296734776f1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7d3ab2ba41e9b73f83f630db07dbaff6" ns2:_="" ns3:_="">
     <xsd:import namespace="f34ab2e2-b096-4083-affb-0a831dd0603a"/>
@@ -1137,27 +1174,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BCFE7A1-554B-47F6-91ED-4FB1C6EB63F5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e72a1ac6-4952-47dd-a4df-3296734776f1"/>
+    <ds:schemaRef ds:uri="f34ab2e2-b096-4083-affb-0a831dd0603a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="e72a1ac6-4952-47dd-a4df-3296734776f1" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f34ab2e2-b096-4083-affb-0a831dd0603a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF96BC3B-6585-4A1C-B15C-D92C6C4D249C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D178728-E33D-441A-B9DF-4CAFBB6B0735}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1174,23 +1210,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF96BC3B-6585-4A1C-B15C-D92C6C4D249C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BCFE7A1-554B-47F6-91ED-4FB1C6EB63F5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e72a1ac6-4952-47dd-a4df-3296734776f1"/>
-    <ds:schemaRef ds:uri="f34ab2e2-b096-4083-affb-0a831dd0603a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>